<commit_message>
Bill: 180 kg-cm BL51180-24V servo, 10 A fuses, battery isolator switches
Steering needed a firm push, so the 60 kg-cm DS5160 + UBEC became the
BL51180-24V (runs from 6S directly). 5 A fuses -> 10 A for the 24 V
servo lead. Two keyed 100 A isolators, one per LiPo. Total Rs 16,295,
matching the Robu cart.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/navya_bill_robu.xlsx
+++ b/docs/navya_bill_robu.xlsx
@@ -90,12 +90,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="130">
   <si>
     <t xml:space="preserve">Navya - Steering &amp; Upgrades Bill (Robu.in)</t>
   </si>
   <si>
-    <t xml:space="preserve">Route A (servo steering) + wiring + e-stop + 256 GB microSD. Prices incl. GST, checked on Robu.in 31-Oct-2026. Blue cells = quantities/prices you can change; totals update.</t>
+    <t xml:space="preserve">Route A (servo steering) + wiring + e-stop + battery switches + 256 GB microSD. Prices incl. GST, checked on Robu.in 31-Oct-2026. Blue cells = quantities/prices you can change; totals update.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -137,10 +137,10 @@
     <t xml:space="preserve">Steering servo</t>
   </si>
   <si>
-    <t xml:space="preserve">Pro-Range DS5160 60kg·cm Metal Gear Digital Servo Motor - 180°</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R251566</t>
+    <t xml:space="preserve">Pro-Range Brushless BL51180-24V 180kg·cm Metal Gear Digital Servo - 180°</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R251585</t>
   </si>
   <si>
     <t xml:space="preserve">In stock</t>
@@ -149,7 +149,7 @@
     <t xml:space="preserve">Open</t>
   </si>
   <si>
-    <t xml:space="preserve">Turns the front axle. 60 kg·cm, 6-8.4 V, metal gears, 25T spline. Replaces the zip tie.</t>
+    <t xml:space="preserve">Turns the front axle. 165-205 kg·cm; runs on 19.2-25.2 V = straight from the 6S LiPo (no UBEC). Chosen over the 60 kg·cm DS5160 because the steering needs a firm push and must cope with roads.</t>
   </si>
   <si>
     <t xml:space="preserve">Servo arm</t>
@@ -161,19 +161,7 @@
     <t xml:space="preserve">28414</t>
   </si>
   <si>
-    <t xml:space="preserve">Connects the servo to the steering link. Check the 25T fit on arrival.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Servo power supply</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ubec-8A 6-36V 2~8S</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1295647</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Powers the servo from a 6S LiPo (25.2 V full). Set output to 7.4 V. 8 A continuous, 15 A peak.</t>
+    <t xml:space="preserve">Connects the servo to the steering link. Check the spline fit on arrival.</t>
   </si>
   <si>
     <t xml:space="preserve">Ball joints (rod ends)</t>
@@ -242,16 +230,16 @@
     <t xml:space="preserve">Inline fuse on the servo / steering power lead.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuses 5 A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Littelfuse 0287005.PXCN Blade Fuse 5A 32V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R182196</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 A fuse for the servo lead, plus spares.</t>
+    <t xml:space="preserve">Fuses 10 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Littelfuse 0287010.PXCN Blade Fuse 10A 32V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R182177</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 A fuse for the 24 V servo lead (a 5 A fuse could blow when the servo pushes hard), plus spares.</t>
   </si>
   <si>
     <t xml:space="preserve">LiPo tap (male)</t>
@@ -341,6 +329,33 @@
     <t xml:space="preserve">Socket with wires for the relay.</t>
   </si>
   <si>
+    <t xml:space="preserve">Battery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main switch, left battery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12V/24V Battery Disconnect Isolator Switch 100A, Red + 2 keys + 4 copper rings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R265245</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key switch in the left LiPo's + lead: turn off instead of unplugging at the controller. 100 A continuous.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main switch, right battery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12V/24V Battery Disconnect Isolator Switch 100A, Black + 2 keys + 4 copper rings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R265246</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same for the right LiPo. Two separate switches keep the batteries separate (never joined).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Storage</t>
   </si>
   <si>
@@ -365,6 +380,9 @@
     <t xml:space="preserve">Safety subtotal</t>
   </si>
   <si>
+    <t xml:space="preserve">Battery subtotal</t>
+  </si>
+  <si>
     <t xml:space="preserve">Storage subtotal</t>
   </si>
   <si>
@@ -422,7 +440,16 @@
     <t xml:space="preserve">Choices and alternatives</t>
   </si>
   <si>
-    <t xml:space="preserve">Servo bracket: Robu has no bracket for the large DS5160 (about 65 x 30 x 48 mm). Make one from aluminium angle or 3D-print it.</t>
+    <t xml:space="preserve">Servo: upgraded from DS5160 60 kg·cm (₹2,329 + ₹1,829 UBEC) to BL51180-24V 180 kg·cm (₹7,329, no UBEC) after the</t>
+  </si>
+  <si>
+    <t xml:space="preserve">steering-effort test needed a firm push. 150/160 kg·cm servos (DS51150-12V, DS51160-24V) were out of stock.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servo bracket: Robu has no bracket for this large servo class (about 65 x 30 x 48 mm). Make one from aluminium angle or 3D-print it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery switches: 1-2-BOTH selector switches were avoided on purpose; they join both LiPos, which is unsafe if their charge differs.</t>
   </si>
   <si>
     <t xml:space="preserve">Link rod: Robu has no M4 threaded rod, so M4 male-female brass standoffs are screwed together into an adjustable rod.</t>
@@ -434,9 +461,6 @@
     <t xml:space="preserve">256 GB card for heavy, continuous recording: SanDisk V30 256GB High Endurance (SKU R165746, ₹7,699, in stock).</t>
   </si>
   <si>
-    <t xml:space="preserve">UBEC: the cheaper 'UBEC-8A DC-DC voltage regulator' (SKU 1345195, ₹1,149) has the same specs but was OUT OF STOCK.</t>
-  </si>
-  <si>
     <t xml:space="preserve">E-stop relay + socket (₹389) are optional if the e-stop is wired in series with both controllers' power-lock wires.</t>
   </si>
   <si>
@@ -446,13 +470,10 @@
     <t xml:space="preserve">Before ordering</t>
   </si>
   <si>
-    <t xml:space="preserve">Remove the steering zip tie and turn the front wheels by hand. Easy: 60 kg·cm servo is fine. Stiff: consider</t>
-  </si>
-  <si>
-    <t xml:space="preserve">the Pro-Range DS51160-24V 160 kg·cm servo (SKU R251583, ₹3,139), which needs a 24 V-rated supply check.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Route A needs the toy steering gearbox disconnected from the linkage, otherwise the servo fights it.</t>
+    <t xml:space="preserve">Done: steering-effort test (needs a firm push) -&gt; 180 kg·cm servo chosen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route A needs the toy steering gearbox disconnected from the linkage, otherwise the servo fights it. Grease the pivots.</t>
   </si>
   <si>
     <t xml:space="preserve">Wiring change with a servo (handled in firmware)</t>
@@ -1011,7 +1032,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -1071,7 +1092,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -1091,11 +1112,11 @@
         <v>1</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>2329</v>
+        <v>7329</v>
       </c>
       <c r="H5" s="7" t="n">
         <f aca="false">F5*G5</f>
-        <v>2329</v>
+        <v>7329</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>17</v>
@@ -1163,11 +1184,11 @@
         <v>1</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>1829</v>
+        <v>299</v>
       </c>
       <c r="H7" s="7" t="n">
         <f aca="false">F7*G7</f>
-        <v>1829</v>
+        <v>299</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>17</v>
@@ -1199,11 +1220,11 @@
         <v>1</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>299</v>
+        <v>167</v>
       </c>
       <c r="H8" s="7" t="n">
         <f aca="false">F8*G8</f>
-        <v>299</v>
+        <v>167</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>17</v>
@@ -1216,83 +1237,83 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>167</v>
-      </c>
-      <c r="H9" s="7" t="n">
+      <c r="G9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="12" t="n">
         <f aca="false">F9*G9</f>
-        <v>167</v>
-      </c>
-      <c r="I9" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <f aca="false">F10*G10</f>
+        <v>46</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K9" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="12" t="n">
-        <f aca="false">F10*G10</f>
-        <v>0</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="J10" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="K10" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K10" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>42</v>
@@ -1304,14 +1325,14 @@
         <v>44</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>23</v>
+        <v>629</v>
       </c>
       <c r="H11" s="7" t="n">
         <f aca="false">F11*G11</f>
-        <v>46</v>
+        <v>629</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>17</v>
@@ -1323,12 +1344,12 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>46</v>
@@ -1340,14 +1361,14 @@
         <v>48</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>629</v>
+        <v>17</v>
       </c>
       <c r="H12" s="7" t="n">
         <f aca="false">F12*G12</f>
-        <v>629</v>
+        <v>68</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>17</v>
@@ -1364,7 +1385,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>50</v>
@@ -1376,14 +1397,14 @@
         <v>52</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>14</v>
+        <v>89</v>
       </c>
       <c r="H13" s="7" t="n">
         <f aca="false">F13*G13</f>
-        <v>56</v>
+        <v>89</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>17</v>
@@ -1400,7 +1421,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>54</v>
@@ -1415,11 +1436,11 @@
         <v>1</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="H14" s="7" t="n">
         <f aca="false">F14*G14</f>
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>17</v>
@@ -1436,7 +1457,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>58</v>
@@ -1448,14 +1469,14 @@
         <v>60</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="H15" s="7" t="n">
         <f aca="false">F15*G15</f>
-        <v>74</v>
+        <v>114</v>
       </c>
       <c r="I15" s="4" t="s">
         <v>17</v>
@@ -1472,7 +1493,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>62</v>
@@ -1503,31 +1524,31 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>57</v>
+        <v>1071</v>
       </c>
       <c r="H17" s="7" t="n">
         <f aca="false">F17*G17</f>
-        <v>114</v>
+        <v>1071</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>17</v>
@@ -1536,15 +1557,15 @@
         <v>18</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>71</v>
@@ -1559,11 +1580,11 @@
         <v>1</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>1071</v>
+        <v>170</v>
       </c>
       <c r="H18" s="7" t="n">
         <f aca="false">F18*G18</f>
-        <v>1071</v>
+        <v>170</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>17</v>
@@ -1575,12 +1596,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
         <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>75</v>
@@ -1595,11 +1616,11 @@
         <v>1</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>170</v>
+        <v>219</v>
       </c>
       <c r="H19" s="7" t="n">
         <f aca="false">F19*G19</f>
-        <v>170</v>
+        <v>219</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>17</v>
@@ -1616,26 +1637,26 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>219</v>
+        <v>909</v>
       </c>
       <c r="H20" s="7" t="n">
         <f aca="false">F20*G20</f>
-        <v>219</v>
+        <v>909</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>17</v>
@@ -1644,7 +1665,7 @@
         <v>18</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1652,7 +1673,7 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>84</v>
@@ -1667,11 +1688,11 @@
         <v>1</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>3999</v>
+        <v>909</v>
       </c>
       <c r="H21" s="7" t="n">
         <f aca="false">F21*G21</f>
-        <v>3999</v>
+        <v>909</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>17</v>
@@ -1683,54 +1704,99 @@
         <v>87</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G23" s="13" t="s">
+    <row r="22" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="H23" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$21,"Steering",$H$5:$H$21)</f>
-        <v>4713</v>
+      <c r="C22" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>3999</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <f aca="false">F22*G22</f>
+        <v>3999</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G24" s="13" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H24" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$21,"Wiring",$H$5:$H$21)</f>
-        <v>1122</v>
+        <f aca="false">SUMIF($B$5:$B$22,"Steering",$H$5:$H$22)</f>
+        <v>7884</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G25" s="13" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H25" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$21,"Safety",$H$5:$H$21)</f>
-        <v>1460</v>
+        <f aca="false">SUMIF($B$5:$B$22,"Wiring",$H$5:$H$22)</f>
+        <v>1134</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G26" s="13" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H26" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$21,"Storage",$H$5:$H$21)</f>
+        <f aca="false">SUMIF($B$5:$B$22,"Safety",$H$5:$H$22)</f>
+        <v>1460</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G27" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <f aca="false">SUMIF($B$5:$B$22,"Battery",$H$5:$H$22)</f>
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G28" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <f aca="false">SUMIF($B$5:$B$22,"Storage",$H$5:$H$22)</f>
         <v>3999</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G27" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="H27" s="16" t="n">
-        <f aca="false">SUM(H5:H21)</f>
-        <v>11294</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G28" s="2" t="s">
-        <v>93</v>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G29" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="H29" s="16" t="n">
+        <f aca="false">SUM(H5:H22)</f>
+        <v>16295</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G30" s="2" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1739,7 +1805,7 @@
     <hyperlink ref="J6" r:id="rId3" display="Open"/>
     <hyperlink ref="J7" r:id="rId4" display="Open"/>
     <hyperlink ref="J8" r:id="rId5" display="Open"/>
-    <hyperlink ref="J9" r:id="rId6" display="Open"/>
+    <hyperlink ref="J10" r:id="rId6" display="Open"/>
     <hyperlink ref="J11" r:id="rId7" display="Open"/>
     <hyperlink ref="J12" r:id="rId8" display="Open"/>
     <hyperlink ref="J13" r:id="rId9" display="Open"/>
@@ -1751,6 +1817,7 @@
     <hyperlink ref="J19" r:id="rId15" display="Open"/>
     <hyperlink ref="J20" r:id="rId16" display="Open"/>
     <hyperlink ref="J21" r:id="rId17" display="Open"/>
+    <hyperlink ref="J22" r:id="rId18" display="Open"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1759,7 +1826,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId18"/>
+  <legacyDrawing r:id="rId19"/>
 </worksheet>
 </file>
 
@@ -1785,12 +1852,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1833,16 +1900,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>1</v>
@@ -1861,7 +1928,7 @@
         <v>18</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1869,16 +1936,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>1</v>
@@ -1897,12 +1964,12 @@
         <v>18</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G8" s="13" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="H8" s="14" t="n">
         <f aca="false">SUMIF($B$5:$B$6,"Steering (alt.)",$H$5:$H$6)</f>
@@ -1911,7 +1978,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G9" s="15" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H9" s="16" t="n">
         <f aca="false">SUM(H5:H6)</f>
@@ -1920,7 +1987,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G10" s="2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1944,7 +2011,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="130"/>
@@ -1952,7 +2019,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1960,12 +2027,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1973,78 +2040,83 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
+      <c r="A14" s="17" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
-        <v>117</v>
+      <c r="A15" s="17" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
-        <v>118</v>
-      </c>
+      <c r="A16" s="17"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>119</v>
+      <c r="A17" s="18" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17"/>
+      <c r="A19" s="17" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
-        <v>121</v>
-      </c>
+      <c r="A20" s="17"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
-        <v>122</v>
+      <c r="A21" s="18" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="17" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bill: keep the toy steering (professor's decision), mark what the current car needs
Adds the BTS7960 driver and a 10k steering-angle potentiometer for the
toy's own steering motor. Servo-conversion rows are kept but marked 'No'.
Needed for the current car: Rs 9,742; servo items not needed: Rs 7,884.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/navya_bill_robu.xlsx
+++ b/docs/navya_bill_robu.xlsx
@@ -90,12 +90,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="151">
   <si>
     <t xml:space="preserve">Navya - Steering &amp; Upgrades Bill (Robu.in)</t>
   </si>
   <si>
-    <t xml:space="preserve">Route A (servo steering) + wiring + e-stop + battery switches + 256 GB microSD. Prices incl. GST, checked on Robu.in 31-Oct-2026. Blue cells = quantities/prices you can change; totals update.</t>
+    <t xml:space="preserve">Professor's decision: keep the toy's own steering. Column L marks what the CURRENT car needs (Yes); servo-conversion rows are kept but marked No. Prices incl. GST, checked on Robu.in 31-Oct-2026. Blue cells = quantities/prices you can change; totals update.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -131,6 +131,45 @@
     <t xml:space="preserve">Why we need it</t>
   </si>
   <si>
+    <t xml:space="preserve">Needed for current car?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toy steering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steering motor driver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SmartElex BTS7960 DC Motor Driver Module (43 A, 6-27 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R189064</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADDED for the current car: lets the Arduino drive the toy's own steering motor left/right with PWM. Powered from the car's existing 12 V battery.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steering angle sensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10K Ohm 3Pin 15mm Shaft Potentiometer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">607345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADDED for the current car: coupled to the steering shaft so the Arduino knows the wheel angle (the toy motor has no sensor). Qty 2 = one spare.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Steering</t>
   </si>
   <si>
@@ -143,15 +182,12 @@
     <t xml:space="preserve">R251585</t>
   </si>
   <si>
-    <t xml:space="preserve">In stock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open</t>
-  </si>
-  <si>
     <t xml:space="preserve">Turns the front axle. 165-205 kg·cm; runs on 19.2-25.2 V = straight from the 6S LiPo (no UBEC). Chosen over the 60 kg·cm DS5160 because the steering needs a firm push and must cope with roads.</t>
   </si>
   <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
     <t xml:space="preserve">Servo arm</t>
   </si>
   <si>
@@ -371,6 +407,9 @@
     <t xml:space="preserve">Trip recordings (about 16 h of video). Kingston 256GB (₹1,853) is out of stock; see Notes.</t>
   </si>
   <si>
+    <t xml:space="preserve">Toy steering subtotal</t>
+  </si>
+  <si>
     <t xml:space="preserve">Steering subtotal</t>
   </si>
   <si>
@@ -386,13 +425,19 @@
     <t xml:space="preserve">Storage subtotal</t>
   </si>
   <si>
-    <t xml:space="preserve">GRAND TOTAL</t>
+    <t xml:space="preserve">GRAND TOTAL (all rows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEEDED FOR CURRENT CAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servo-conversion items (not needed now)</t>
   </si>
   <si>
     <t xml:space="preserve">Shipping (if any) is extra; Robu shows it at checkout.</t>
   </si>
   <si>
-    <t xml:space="preserve">Route B - keep the toy steering motor (instead of Bill rows 1-6)</t>
+    <t xml:space="preserve">Route B - keep the toy steering motor (now chosen: see 'Toy steering' rows on the Bill sheet)</t>
   </si>
   <si>
     <t xml:space="preserve">Cheaper parts but more work: the sensor must be fitted to the steering shaft and the Arduino runs the position loop. Power from the car's existing 12 V battery.</t>
@@ -407,9 +452,6 @@
     <t xml:space="preserve">SmartElex BTS7960 DC Motor Driver Module</t>
   </si>
   <si>
-    <t xml:space="preserve">R189064</t>
-  </si>
-  <si>
     <t xml:space="preserve">Drives the toy's own steering motor both ways. The cheaper 'Double BTS7960' (₹329) is out of stock.</t>
   </si>
   <si>
@@ -435,6 +477,27 @@
   </si>
   <si>
     <t xml:space="preserve">Prices and stock change often; open each link and recheck before paying.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision (31-Oct-2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Professor: do not change the steering; work with the toy's own steering motor and gearbox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">So the car needs a motor driver (BTS7960) and an angle sensor (10k potentiometer on the steering shaft).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servo, servo arm, ball joints, link standoffs and bracket stay in the bill for reference, marked 'No'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toy steering motor power: the car's existing 12 V battery (no purchase). Arduino: driver RPWM/LPWM on two PWM pins,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">potentiometer on A0, limit switches on two digital pins; brakes move off D5/D6 (handled in firmware).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AS5600 magnetic sensor (SKU R175153, ₹159) is an alternative to the potentiometer, but Robu's module comes WITHOUT the magnet.</t>
   </si>
   <si>
     <t xml:space="preserve">Choices and alternatives</t>
@@ -570,7 +633,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -585,14 +648,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -645,7 +720,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -682,19 +757,27 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -706,12 +789,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -766,8 +861,8 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -1032,11 +1127,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
@@ -1045,6 +1140,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1091,113 +1187,125 @@
       <c r="K4" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="46" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L4" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>7329</v>
+        <v>1273</v>
       </c>
       <c r="H5" s="7" t="n">
         <f aca="false">F5*G5</f>
-        <v>7329</v>
+        <v>1273</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>20</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>89</v>
+        <v>29</v>
       </c>
       <c r="H6" s="7" t="n">
         <f aca="false">F6*G6</f>
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>25</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="46" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>299</v>
+        <v>7329</v>
       </c>
       <c r="H7" s="7" t="n">
         <f aca="false">F7*G7</f>
-        <v>299</v>
+        <v>7329</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+      <c r="L7" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1205,71 +1313,77 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>167</v>
+        <v>89</v>
       </c>
       <c r="H8" s="7" t="n">
         <f aca="false">F8*G8</f>
-        <v>167</v>
+        <v>89</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L8" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>299</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <f aca="false">F9*G9</f>
+        <v>299</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="J9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L9" s="10" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="12" t="n">
-        <f aca="false">F9*G9</f>
-        <v>0</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1277,71 +1391,77 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>23</v>
+        <v>167</v>
       </c>
       <c r="H10" s="7" t="n">
         <f aca="false">F10*G10</f>
+        <v>167</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="6" t="n">
-        <v>629</v>
-      </c>
-      <c r="H11" s="7" t="n">
+      <c r="G11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14" t="n">
         <f aca="false">F11*G11</f>
-        <v>629</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>45</v>
+        <v>0</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="J11" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="L11" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1349,35 +1469,38 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H12" s="7" t="n">
         <f aca="false">F12*G12</f>
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1385,71 +1508,77 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>89</v>
+        <v>629</v>
       </c>
       <c r="H13" s="7" t="n">
         <f aca="false">F13*G13</f>
-        <v>89</v>
+        <v>629</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>57</v>
+      </c>
+      <c r="L13" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="H14" s="7" t="n">
         <f aca="false">F14*G14</f>
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>57</v>
+        <v>61</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1457,35 +1586,38 @@
         <v>11</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>57</v>
+        <v>89</v>
       </c>
       <c r="H15" s="7" t="n">
         <f aca="false">F15*G15</f>
-        <v>114</v>
+        <v>89</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>61</v>
+        <v>65</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1493,107 +1625,116 @@
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="H16" s="7" t="n">
         <f aca="false">F16*G16</f>
-        <v>114</v>
+        <v>74</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>69</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
         <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>1071</v>
+        <v>57</v>
       </c>
       <c r="H17" s="7" t="n">
         <f aca="false">F17*G17</f>
-        <v>1071</v>
+        <v>114</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>73</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>170</v>
+        <v>57</v>
       </c>
       <c r="H18" s="7" t="n">
         <f aca="false">F18*G18</f>
-        <v>170</v>
+        <v>114</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
+      </c>
+      <c r="L18" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1601,71 +1742,77 @@
         <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>219</v>
+        <v>1071</v>
       </c>
       <c r="H19" s="7" t="n">
         <f aca="false">F19*G19</f>
-        <v>219</v>
+        <v>1071</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>82</v>
+      </c>
+      <c r="L19" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>909</v>
+        <v>170</v>
       </c>
       <c r="H20" s="7" t="n">
         <f aca="false">F20*G20</f>
-        <v>909</v>
+        <v>170</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
+      </c>
+      <c r="L20" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1673,35 +1820,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>909</v>
+        <v>219</v>
       </c>
       <c r="H21" s="7" t="n">
         <f aca="false">F21*G21</f>
-        <v>909</v>
+        <v>219</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1709,94 +1859,202 @@
         <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>3999</v>
+        <v>909</v>
       </c>
       <c r="H22" s="7" t="n">
         <f aca="false">F22*G22</f>
+        <v>909</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>909</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <f aca="false">F23*G23</f>
+        <v>909</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="L23" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="6" t="n">
         <v>3999</v>
       </c>
-      <c r="I22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J22" s="8" t="s">
+      <c r="H24" s="7" t="n">
+        <f aca="false">F24*G24</f>
+        <v>3999</v>
+      </c>
+      <c r="I24" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="K22" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G24" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="H24" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$22,"Steering",$H$5:$H$22)</f>
+      <c r="J24" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="L24" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G26" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <f aca="false">SUMIF($B$5:$B$24,"Toy steering",$H$5:$H$24)</f>
+        <v>1331</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G27" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <f aca="false">SUMIF($B$5:$B$24,"Steering",$H$5:$H$24)</f>
         <v>7884</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G25" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="H25" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$22,"Wiring",$H$5:$H$22)</f>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G28" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="H28" s="16" t="n">
+        <f aca="false">SUMIF($B$5:$B$24,"Wiring",$H$5:$H$24)</f>
         <v>1134</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G26" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="H26" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$22,"Safety",$H$5:$H$22)</f>
-        <v>1460</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G27" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="H27" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$22,"Battery",$H$5:$H$22)</f>
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G28" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="H28" s="14" t="n">
-        <f aca="false">SUMIF($B$5:$B$22,"Storage",$H$5:$H$22)</f>
-        <v>3999</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G29" s="15" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="H29" s="16" t="n">
-        <f aca="false">SUM(H5:H22)</f>
-        <v>16295</v>
+        <f aca="false">SUMIF($B$5:$B$24,"Safety",$H$5:$H$24)</f>
+        <v>1460</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G30" s="2" t="s">
-        <v>99</v>
+      <c r="G30" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="H30" s="16" t="n">
+        <f aca="false">SUMIF($B$5:$B$24,"Battery",$H$5:$H$24)</f>
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G31" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="H31" s="16" t="n">
+        <f aca="false">SUMIF($B$5:$B$24,"Storage",$H$5:$H$24)</f>
+        <v>3999</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G32" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="H32" s="18" t="n">
+        <f aca="false">SUM(H5:H24)</f>
+        <v>17626</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G33" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="H33" s="20" t="n">
+        <f aca="false">SUMIF($L$5:$L$24,"Yes",$H$5:$H$24)</f>
+        <v>9742</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G34" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="H34" s="16" t="n">
+        <f aca="false">SUMIF($L$5:$L$24,"No",$H$5:$H$24)</f>
+        <v>7884</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G35" s="2" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1805,8 +2063,8 @@
     <hyperlink ref="J6" r:id="rId3" display="Open"/>
     <hyperlink ref="J7" r:id="rId4" display="Open"/>
     <hyperlink ref="J8" r:id="rId5" display="Open"/>
-    <hyperlink ref="J10" r:id="rId6" display="Open"/>
-    <hyperlink ref="J11" r:id="rId7" display="Open"/>
+    <hyperlink ref="J9" r:id="rId6" display="Open"/>
+    <hyperlink ref="J10" r:id="rId7" display="Open"/>
     <hyperlink ref="J12" r:id="rId8" display="Open"/>
     <hyperlink ref="J13" r:id="rId9" display="Open"/>
     <hyperlink ref="J14" r:id="rId10" display="Open"/>
@@ -1818,6 +2076,8 @@
     <hyperlink ref="J20" r:id="rId16" display="Open"/>
     <hyperlink ref="J21" r:id="rId17" display="Open"/>
     <hyperlink ref="J22" r:id="rId18" display="Open"/>
+    <hyperlink ref="J23" r:id="rId19" display="Open"/>
+    <hyperlink ref="J24" r:id="rId20" display="Open"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1826,7 +2086,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId19"/>
+  <legacyDrawing r:id="rId21"/>
 </worksheet>
 </file>
 
@@ -1835,11 +2095,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
@@ -1848,16 +2108,17 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1894,22 +2155,25 @@
       <c r="K4" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="L4" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>105</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>1</v>
@@ -1922,13 +2186,16 @@
         <v>1273</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>106</v>
+        <v>120</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1936,16 +2203,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>1</v>
@@ -1958,36 +2225,57 @@
         <v>159</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>110</v>
+        <v>124</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G8" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="H8" s="14" t="n">
+      <c r="G8" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="H8" s="16" t="n">
         <f aca="false">SUMIF($B$5:$B$6,"Steering (alt.)",$H$5:$H$6)</f>
         <v>1432</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G9" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="H9" s="16" t="n">
+      <c r="G9" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="H9" s="18" t="n">
         <f aca="false">SUM(H5:H6)</f>
         <v>1432</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G10" s="2" t="s">
-        <v>99</v>
+      <c r="G10" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <f aca="false">SUMIF($L$5:$L$6,"Yes",$H$5:$H$6)</f>
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G11" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <f aca="false">SUMIF($L$5:$L$6,"No",$H$5:$H$6)</f>
+        <v>159</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G12" s="2" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -2011,7 +2299,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="130"/>
@@ -2019,104 +2307,142 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17"/>
+      <c r="A2" s="22"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="17" t="s">
-        <v>113</v>
+      <c r="A3" s="22" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
-        <v>114</v>
+      <c r="A4" s="22" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17"/>
+      <c r="A5" s="22"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
-        <v>115</v>
+      <c r="A6" s="23" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>116</v>
+      <c r="A7" s="22" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>117</v>
+      <c r="A8" s="22" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>118</v>
+      <c r="A9" s="22" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>119</v>
+      <c r="A10" s="22" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>120</v>
+      <c r="A11" s="22" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
-        <v>121</v>
+      <c r="A12" s="22" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
-        <v>122</v>
-      </c>
+      <c r="A13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
-        <v>123</v>
+      <c r="A14" s="23" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
-        <v>124</v>
+      <c r="A15" s="22" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17"/>
+      <c r="A16" s="22" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
-        <v>125</v>
+      <c r="A17" s="22" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
-        <v>126</v>
+      <c r="A18" s="22" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>127</v>
+      <c r="A19" s="22" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
+      <c r="A20" s="22" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
-        <v>128</v>
+      <c r="A21" s="22" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
-        <v>129</v>
+      <c r="A22" s="22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="22" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="22"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="23" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="22" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="22" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="22"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="23" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="22" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>